<commit_message>
v5: top-centred title, decluttered layout, zero overlaps (supersedes v4)
</commit_message>
<xml_diff>
--- a/KAMIL BHAI WORK/MRM_Master_Data.xlsx
+++ b/KAMIL BHAI WORK/MRM_Master_Data.xlsx
@@ -436,19 +436,19 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Variance vs Baseline</t>
+          <t>Var vs BL %</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Gap (Cr)</t>
+          <t>Gap Cr</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FTM (This Month)</t>
+          <t>FTM</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -472,7 +472,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CUM (Inception to Date)</t>
+          <t>CUM</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -570,7 +570,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -583,7 +583,7 @@
         <v>1691</v>
       </c>
       <c r="C3" t="n">
-        <v>2000</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="4">
@@ -620,30 +620,6 @@
       </c>
       <c r="B6" t="n">
         <v>344498</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>WIR C/O</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>118 / 26</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>MIR C/O</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>63 / 1</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v7: full-deck redesign (slides 5-38), type scale stepped down ~10%
- New output MRM_Aug-26_Redesigned_V7.pptx; master pptx untouched (md5 verified)
- Slides 1-4 unchanged; 5-38 rebuilt on the v7 design system
- Heading and body type reduced ~10%; titles auto-shrink to clear the logo band
- 21 charts, all embedded-workbook linked; 7 SharePoint-linked charts (incl. the 3-D one) removed
- Photo slides re-harvested, de-chromed, cropped to a regular grid and captioned
- Hidden original slide 9 (BIM clash) restored to visible
- Stale relationships pruned, shape ids renumbered, 0 off-canvas, 0 text overlaps
- validate.py and qa.py both PASS; 38/38 pages rendered and reviewed
- Adds V7_BUILD_NOTES.md, V7_Renders/ and src/; retires the V6 slide-5 artifacts
</commit_message>
<xml_diff>
--- a/KAMIL BHAI WORK/MRM_Master_Data.xlsx
+++ b/KAMIL BHAI WORK/MRM_Master_Data.xlsx
@@ -10,6 +10,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Commercial" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Safety" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BIM" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clash" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Constr" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manpower" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SeptPlan" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EHS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualityInd" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -498,6 +506,228 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>FTM</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ITD</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Safe Manhours</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>127954</v>
+      </c>
+      <c r="C2" t="n">
+        <v>344498</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Inductions</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>585</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Training Sessions</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tool Box Talks</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>265</v>
+      </c>
+      <c r="C5" t="n">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Safety Observations</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>122</v>
+      </c>
+      <c r="C6" t="n">
+        <v>781</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Lagging</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Training Imparted</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>74</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Obs. External</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Good/Best Practices</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Obs. Internal</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Material Approvals</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Rejection</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Management Walkdown</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Repetitive Dev.</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Mockups</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Snag Issued</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Stop Work</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -625,4 +855,499 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DD Approved</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1014</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1220</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GFC Approved</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>178</v>
+      </c>
+      <c r="C3" t="n">
+        <v>247</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Structure</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>MEPF</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>BOH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Substructure</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>84</v>
+      </c>
+      <c r="C2" t="n">
+        <v>80</v>
+      </c>
+      <c r="D2" t="n">
+        <v>82</v>
+      </c>
+      <c r="E2" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3H Hotel</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>83</v>
+      </c>
+      <c r="C3" t="n">
+        <v>82</v>
+      </c>
+      <c r="D3" t="n">
+        <v>86</v>
+      </c>
+      <c r="E3" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4H Hotel</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>82</v>
+      </c>
+      <c r="C4" t="n">
+        <v>81</v>
+      </c>
+      <c r="D4" t="n">
+        <v>84</v>
+      </c>
+      <c r="E4" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Retail 1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>86</v>
+      </c>
+      <c r="C5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D5" t="n">
+        <v>83</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Retail 2</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>86</v>
+      </c>
+      <c r="C6" t="n">
+        <v>83</v>
+      </c>
+      <c r="D6" t="n">
+        <v>86</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Convention</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>83</v>
+      </c>
+      <c r="C7" t="n">
+        <v>85</v>
+      </c>
+      <c r="D7" t="n">
+        <v>86</v>
+      </c>
+      <c r="E7" t="n">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total Clashes</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Hotspot</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>17 Aug</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>15297</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MEPF vs AR</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5131</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>24 Aug</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>34845</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>LA vs MEPF</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2233</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>27 Aug</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>17400</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>MEPF vs ST</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1957</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AR vs ST</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1576</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LA vs ST</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1339</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LA vs LA</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1073</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Concrete m3</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>4-H</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>39</v>
+      </c>
+      <c r="C2" t="n">
+        <v>46</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>3025</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5584</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3-H</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C3" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Workmen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sept Plan</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1205</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>₹ Cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Supply</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>